<commit_message>
fix card disapper after relaoding
</commit_message>
<xml_diff>
--- a/stickers_to_import.xlsx
+++ b/stickers_to_import.xlsx
@@ -1,41 +1,137 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr codeName="ThisWorkbook"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\fadi\Desktop\happy-helper-main\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{661B0A6B-1151-44CC-A9C3-22CE19B1CB6A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <bookViews>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+  </bookViews>
   <sheets>
     <sheet name="Stickers" sheetId="1" r:id="rId1"/>
   </sheets>
+  <calcPr calcId="0"/>
 </workbook>
 </file>
 
-<file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
-<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xlrd="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
-  <metadataTypes count="1">
-    <metadataType name="XLDAPR" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1" cellMeta="1"/>
-  </metadataTypes>
-  <futureMetadata name="XLDAPR" count="1">
-    <bk>
-      <extLst>
-        <ext uri="{bdbb8cdc-fa1e-496e-a857-3c3f30c029c3}">
-          <xda:dynamicArrayProperties fDynamic="1" fCollapsed="0"/>
-        </ext>
-      </extLst>
-    </bk>
-  </futureMetadata>
-  <cellMetadata count="1">
-    <bk>
-      <rc t="1" v="0"/>
-    </bk>
-  </cellMetadata>
-</metadata>
+<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="45" uniqueCount="35">
+  <si>
+    <t>name</t>
+  </si>
+  <si>
+    <t>price</t>
+  </si>
+  <si>
+    <t>category</t>
+  </si>
+  <si>
+    <t>img</t>
+  </si>
+  <si>
+    <t>badge</t>
+  </si>
+  <si>
+    <t>Chopper</t>
+  </si>
+  <si>
+    <t>Anime, One Piece</t>
+  </si>
+  <si>
+    <t>One Piece</t>
+  </si>
+  <si>
+    <t>Chopper Hat</t>
+  </si>
+  <si>
+    <t>Naruto Ramen</t>
+  </si>
+  <si>
+    <t>Anime, Naruto</t>
+  </si>
+  <si>
+    <t>Naruto</t>
+  </si>
+  <si>
+    <t>Anime Girl</t>
+  </si>
+  <si>
+    <t>Anime, Cute</t>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t>Bakugo</t>
+  </si>
+  <si>
+    <t>Anime, My Hero Academia</t>
+  </si>
+  <si>
+    <t>MHA</t>
+  </si>
+  <si>
+    <t>Nanami</t>
+  </si>
+  <si>
+    <t>Anime, Jujutsu Kaisen</t>
+  </si>
+  <si>
+    <t>JJK</t>
+  </si>
+  <si>
+    <t>Megumi Fushiguro</t>
+  </si>
+  <si>
+    <t>Toji Fushiguro</t>
+  </si>
+  <si>
+    <t>Roronoa Zoro</t>
+  </si>
+  <si>
+    <t>One Piece Logo</t>
+  </si>
+  <si>
+    <t>https://i.pinimg.com/1200x/67/2c/ac/672cac0d8d27efb9aa2726c5035c69bc.jpg</t>
+  </si>
+  <si>
+    <t>https://i.pinimg.com/1200x/d5/3f/ea/d53fea51dd433bc36c6a46befd822918.jpg</t>
+  </si>
+  <si>
+    <t>https://i.pinimg.com/736x/7d/52/3d/7d523d2cdaedc9278c3492845b7a0322.jpg</t>
+  </si>
+  <si>
+    <t>https://i.pinimg.com/736x/52/e1/d2/52e1d20ec198670cda0cd93c7565b637.jpg</t>
+  </si>
+  <si>
+    <t>https://i.pinimg.com/736x/1c/1b/65/1c1b6561a8b4c14f7139addb3b3c7c6d.jpg</t>
+  </si>
+  <si>
+    <t>https://i.pinimg.com/736x/7e/97/88/7e9788ed22b898f6bb71c65c6b80aa72.jpg</t>
+  </si>
+  <si>
+    <t>https://i.pinimg.com/1200x/ce/a6/71/cea671eca0d14db693e670ae648d5fb3.jpg</t>
+  </si>
+  <si>
+    <t>https://i.pinimg.com/1200x/5b/46/b4/5b46b4bd27314073c2580be55dc84bcd.jpg</t>
+  </si>
+  <si>
+    <t>https://i.pinimg.com/736x/56/3a/b8/563ab859469b09629e4fd7b0a5f10c87.jpg</t>
+  </si>
+  <si>
+    <t>https://i.pinimg.com/1200x/67/42/ed/6742ed0afda617996339715a3e594687.jpg</t>
+  </si>
+</sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:vt="http://schemas.openxmlformats.org/officeDocument/2006/docPropsVTypes">
-  <numFmts count="1">
-    <numFmt numFmtId="56" formatCode="&quot;上午/下午 &quot;hh&quot;時&quot;mm&quot;分&quot;ss&quot;秒 &quot;"/>
-  </numFmts>
-  <fonts count="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="1" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -65,13 +161,21 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="1">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleMedium4"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
@@ -396,240 +500,208 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F11"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1:E11"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="18.83203125" customWidth="1"/>
-    <col min="2" max="2" width="7.83203125" customWidth="1"/>
-    <col min="3" max="3" width="10.83203125" customWidth="1"/>
-    <col min="4" max="4" width="7.83203125" customWidth="1"/>
-    <col min="5" max="5" width="57.83203125" customWidth="1"/>
-    <col min="6" max="6" width="11.83203125" customWidth="1"/>
+    <col min="1" max="1" width="18.796875" customWidth="1"/>
+    <col min="2" max="2" width="7.796875" customWidth="1"/>
+    <col min="3" max="3" width="25.796875" customWidth="1"/>
+    <col min="4" max="4" width="57.796875" customWidth="1"/>
+    <col min="5" max="5" width="11.796875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1">
-      <c r="A1" t="str">
-        <v>name</v>
-      </c>
-      <c r="B1" t="str">
-        <v>price</v>
-      </c>
-      <c r="C1" t="str">
-        <v>category</v>
-      </c>
-      <c r="D1" t="str">
-        <v>emoji</v>
-      </c>
-      <c r="E1" t="str">
-        <v>img</v>
-      </c>
-      <c r="F1" t="str">
-        <v>badge</v>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="str">
-        <v>Chopper</v>
+    <row r="1" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
+        <v>5</v>
       </c>
       <c r="B2">
         <v>0.5</v>
       </c>
-      <c r="C2" t="str">
-        <v>anime</v>
-      </c>
-      <c r="D2" t="str">
-        <v>🦌</v>
-      </c>
-      <c r="E2" t="str">
-        <v>stickers/WhatsApp Image 2026-04-05 at 00.04.45.jpeg</v>
-      </c>
-      <c r="F2" t="str">
-        <v>One Piece</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="str">
-        <v>Chopper Hat</v>
+      <c r="C2" t="s">
+        <v>6</v>
+      </c>
+      <c r="D2" t="s">
+        <v>25</v>
+      </c>
+      <c r="E2" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
+        <v>8</v>
       </c>
       <c r="B3">
         <v>0.5</v>
       </c>
-      <c r="C3" t="str">
-        <v>anime</v>
-      </c>
-      <c r="D3" t="str">
-        <v>🎩</v>
-      </c>
-      <c r="E3" t="str">
-        <v>stickers/WhatsApp Image 2026-04-05 at 00.04.45 (1).jpeg</v>
-      </c>
-      <c r="F3" t="str">
-        <v>One Piece</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="str">
-        <v>Naruto Ramen</v>
+      <c r="C3" t="s">
+        <v>6</v>
+      </c>
+      <c r="D3" t="s">
+        <v>26</v>
+      </c>
+      <c r="E3" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
+        <v>9</v>
       </c>
       <c r="B4">
         <v>0.5</v>
       </c>
-      <c r="C4" t="str">
-        <v>anime</v>
-      </c>
-      <c r="D4" t="str">
-        <v>🍜</v>
-      </c>
-      <c r="E4" t="str">
-        <v>stickers/WhatsApp Image 2026-04-05 at 00.04.45 (2).jpeg</v>
-      </c>
-      <c r="F4" t="str">
-        <v>Naruto</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="str">
-        <v>Anime Girl</v>
+      <c r="C4" t="s">
+        <v>10</v>
+      </c>
+      <c r="D4" t="s">
+        <v>27</v>
+      </c>
+      <c r="E4" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A5" t="s">
+        <v>12</v>
       </c>
       <c r="B5">
         <v>0.5</v>
       </c>
-      <c r="C5" t="str">
-        <v>anime</v>
-      </c>
-      <c r="D5" t="str">
-        <v>⭐</v>
-      </c>
-      <c r="E5" t="str">
-        <v>stickers/WhatsApp Image 2026-04-05 at 00.04.45 (3).jpeg</v>
-      </c>
-      <c r="F5" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="str">
-        <v>Bakugo</v>
+      <c r="C5" t="s">
+        <v>13</v>
+      </c>
+      <c r="D5" t="s">
+        <v>28</v>
+      </c>
+      <c r="E5" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A6" t="s">
+        <v>15</v>
       </c>
       <c r="B6">
         <v>0.5</v>
       </c>
-      <c r="C6" t="str">
-        <v>anime</v>
-      </c>
-      <c r="D6" t="str">
-        <v>💥</v>
-      </c>
-      <c r="E6" t="str">
-        <v>stickers/WhatsApp Image 2026-04-05 at 00.04.46.jpeg</v>
-      </c>
-      <c r="F6" t="str">
-        <v>MHA</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="str">
-        <v>Nanami</v>
+      <c r="C6" t="s">
+        <v>16</v>
+      </c>
+      <c r="D6" t="s">
+        <v>29</v>
+      </c>
+      <c r="E6" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A7" t="s">
+        <v>18</v>
       </c>
       <c r="B7">
         <v>0.5</v>
       </c>
-      <c r="C7" t="str">
-        <v>anime</v>
-      </c>
-      <c r="D7" t="str">
-        <v>🕴️</v>
-      </c>
-      <c r="E7" t="str">
-        <v>stickers/WhatsApp Image 2026-04-05 at 00.04.46 (1).jpeg</v>
-      </c>
-      <c r="F7" t="str">
-        <v>JJK</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="str">
-        <v>Megumi Fushiguro</v>
+      <c r="C7" t="s">
+        <v>19</v>
+      </c>
+      <c r="D7" t="s">
+        <v>30</v>
+      </c>
+      <c r="E7" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A8" t="s">
+        <v>21</v>
       </c>
       <c r="B8">
         <v>0.5</v>
       </c>
-      <c r="C8" t="str">
-        <v>anime</v>
-      </c>
-      <c r="D8" t="str">
-        <v>🖤</v>
-      </c>
-      <c r="E8" t="str">
-        <v>stickers/WhatsApp Image 2026-04-05 at 00.04.46 (2).jpeg</v>
-      </c>
-      <c r="F8" t="str">
-        <v>JJK</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="str">
-        <v>Toji Fushiguro</v>
+      <c r="C8" t="s">
+        <v>19</v>
+      </c>
+      <c r="D8" t="s">
+        <v>31</v>
+      </c>
+      <c r="E8" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A9" t="s">
+        <v>22</v>
       </c>
       <c r="B9">
         <v>0.5</v>
       </c>
-      <c r="C9" t="str">
-        <v>anime</v>
-      </c>
-      <c r="D9" t="str">
-        <v>👊</v>
-      </c>
-      <c r="E9" t="str">
-        <v>stickers/WhatsApp Image 2026-04-05 at 00.04.46 (3).jpeg</v>
-      </c>
-      <c r="F9" t="str">
-        <v>JJK</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="str">
-        <v>Roronoa Zoro</v>
+      <c r="C9" t="s">
+        <v>19</v>
+      </c>
+      <c r="D9" t="s">
+        <v>32</v>
+      </c>
+      <c r="E9" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A10" t="s">
+        <v>23</v>
       </c>
       <c r="B10">
         <v>0.5</v>
       </c>
-      <c r="C10" t="str">
-        <v>anime</v>
-      </c>
-      <c r="D10" t="str">
-        <v>⚔️</v>
-      </c>
-      <c r="E10" t="str">
-        <v>stickers/WhatsApp Image 2026-04-05 at 00.04.47.jpeg</v>
-      </c>
-      <c r="F10" t="str">
-        <v>One Piece</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="str">
-        <v>One Piece Logo</v>
+      <c r="C10" t="s">
+        <v>6</v>
+      </c>
+      <c r="D10" t="s">
+        <v>33</v>
+      </c>
+      <c r="E10" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A11" t="s">
+        <v>24</v>
       </c>
       <c r="B11">
         <v>0.5</v>
       </c>
-      <c r="C11" t="str">
-        <v>anime</v>
-      </c>
-      <c r="D11" t="str">
-        <v>☠️</v>
-      </c>
-      <c r="E11" t="str">
-        <v>stickers/WhatsApp Image 2026-04-05 at 00.04.47 (1).jpeg</v>
-      </c>
-      <c r="F11" t="str">
-        <v>One Piece</v>
+      <c r="C11" t="s">
+        <v>6</v>
+      </c>
+      <c r="D11" t="s">
+        <v>34</v>
+      </c>
+      <c r="E11" t="s">
+        <v>7</v>
       </c>
     </row>
   </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F11"/>
+    <ignoredError sqref="A1:E1 A11:C11 A2:C2 E2 A3:C3 E3 A4:C4 E4 A5:C5 E5 A6:C6 E6 A7:C7 E7 A8:C8 E8 A9:C9 E9 A10:C10 E10 E11" numberStoredAsText="1"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>